<commit_message>
v2.0: Mejoras en Predicciones
</commit_message>
<xml_diff>
--- a/backend/data/chiki_pronosticos.xlsx
+++ b/backend/data/chiki_pronosticos.xlsx
@@ -36,8 +36,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="4">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="200" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="201" formatCode="yyyy-mm-dd hh:mm"/>
+    <numFmt numFmtId="202" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -402,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:H3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -421,18 +424,12 @@
         <v>rol</v>
       </c>
       <c r="F1" t="str">
-        <v>puntos_iniciales</v>
+        <v>foto_perfil</v>
       </c>
       <c r="G1" t="str">
-        <v>puntos_ganados</v>
+        <v>activo</v>
       </c>
       <c r="H1" t="str">
-        <v>foto_perfil</v>
-      </c>
-      <c r="I1" t="str">
-        <v>activo</v>
-      </c>
-      <c r="J1" t="str">
         <v>creado_en</v>
       </c>
     </row>
@@ -444,136 +441,60 @@
         <v>admin</v>
       </c>
       <c r="C2" t="str">
-        <v>Sergio</v>
+        <v>Sergio Admin</v>
       </c>
       <c r="D2" t="str">
-        <v>d6cbb2e62529c7ec11ab6923884e75ae:ce7fcaae4daf8e451d67d12d4af624ecf4fb8f2efebd1e97732a0c7463e27a4ff4c3831e70c229cd500d70a28f44ce83d9db40e91aa5d4dace4c55fca8c5ae09</v>
+        <v>36b37b42ec5e8946a0e641a5b96e0f2e:172ba8394862537688aea1522a741d1a27379a1827e392e2a343c02b223d6473eec7f6f9c0fb49171708dad15344c2cfe4a75a57e67e41c49036235fbd3a0599</v>
       </c>
       <c r="E2" t="str">
         <v>admin</v>
       </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2" t="str">
-        <v>/uploads/perfiles/3606f96d-d11a-452d-9d69-37888393b4f7.jpg</v>
-      </c>
-      <c r="I2" t="str">
+      <c r="F2" t="str">
+        <v>/uploads/perfiles/00f50d33-3cba-42da-98ea-9d0ae591360d.jpg</v>
+      </c>
+      <c r="G2" t="str">
         <v>si</v>
       </c>
-      <c r="J2">
+      <c r="H2" s="1">
         <v>46186.76034349537</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>9a8be45c-ccde-45b0-9a80-39a0bcbcccf0</v>
+        <v>USR-DEMO-001</v>
       </c>
       <c r="B3" t="str">
-        <v>fabian</v>
+        <v>sergio</v>
       </c>
       <c r="C3" t="str">
-        <v>Fabián Chiquinta</v>
+        <v>Sergio</v>
       </c>
       <c r="D3" t="str">
-        <v>15db4a6af2c6a3042d515579efa43f72:e396890de732e75045c9f5c032fe42bc56addae8577eecbfa03c80e369473d1c8a381abb47f5ae9eb319b72d76e21c155d74d06dff4a30ee02ac9aa701fa4e01</v>
+        <v>401ad1a53866fb30f44f9db6f79527e9:da506aa9e75f82beabb24cfe6274db55f8eea7a5447c800112ed8d39557863084ee64648571630bed3db7111d99ed53c796be8cb0ed489559d5d53f581c2b783</v>
       </c>
       <c r="E3" t="str">
         <v>participante</v>
       </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3" t="str">
+      <c r="F3" t="str">
+        <v>/uploads/perfiles/024cc429-fc92-4951-8fab-af3118629e5a.jpg</v>
+      </c>
+      <c r="G3" t="str">
         <v>si</v>
       </c>
-      <c r="J3" t="str">
-        <v>2026-06-13T18:51:41.620Z</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>19f36595-55b5-4b33-9612-d3794eb78344</v>
-      </c>
-      <c r="B4" t="str">
-        <v>henry</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Henry Chiquinta</v>
-      </c>
-      <c r="D4" t="str">
-        <v>13108c555cf6f5982255ea0f716c5286:9760ffbb7756dda286f1b6a1bfff2e619d48238b089f26855726e7ffe0471f0d5b04f98f8f767cdfe517eda4079f46d8a6c7c4c2d0700e186c2a82dd1bc40775</v>
-      </c>
-      <c r="E4" t="str">
-        <v>participante</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
-      <c r="I4" t="str">
-        <v>si</v>
-      </c>
-      <c r="J4" t="str">
-        <v>2026-06-13T18:52:41.682Z</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>c3e0cf6c-33b8-4e0d-a3f3-5221cb4ebc3e</v>
-      </c>
-      <c r="B5" t="str">
-        <v>sergio</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Sergio Chiquinta</v>
-      </c>
-      <c r="D5" t="str">
-        <v>9ae93c7809ea874147875d3cfb3d800f:7e3e9e8b61ef724ec974ebaba92e31f6889f5ded665c823f3d7856f9558d2a1dce11a4aff030446d6b9b1762f3d3641735c803879ef20f443a297ec088598c0a</v>
-      </c>
-      <c r="E5" t="str">
-        <v>participante</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-      <c r="H5" t="str">
-        <v>/uploads/perfiles/31cee2b8-bbbe-4749-9077-a6413b4f3c9b.jpg</v>
-      </c>
-      <c r="I5" t="str">
-        <v>si</v>
-      </c>
-      <c r="J5" t="str">
-        <v>2026-06-13T18:56:30.418Z</v>
+      <c r="H3" s="1">
+        <v>46186.76034408565</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M105"/>
+  <dimension ref="A1:Q105"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -615,6 +536,18 @@
       <c r="M1" t="str">
         <v>fuente</v>
       </c>
+      <c r="N1" t="str">
+        <v>zona_horaria</v>
+      </c>
+      <c r="O1" t="str">
+        <v>origen_local</v>
+      </c>
+      <c r="P1" t="str">
+        <v>origen_visitante</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>ganador_desempate</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -656,6 +589,18 @@
       <c r="M2" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N2" t="str">
+        <v>America/Mexico_City</v>
+      </c>
+      <c r="O2" t="str">
+        <v>México</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Sudáfrica</v>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -697,6 +642,18 @@
       <c r="M3" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N3" t="str">
+        <v>America/Mexico_City</v>
+      </c>
+      <c r="O3" t="str">
+        <v>Corea del Sur</v>
+      </c>
+      <c r="P3" t="str">
+        <v>Chequia</v>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -738,6 +695,18 @@
       <c r="M4" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N4" t="str">
+        <v>America/Toronto</v>
+      </c>
+      <c r="O4" t="str">
+        <v>Canadá</v>
+      </c>
+      <c r="P4" t="str">
+        <v>Bosnia y Herzegovina</v>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -779,6 +748,18 @@
       <c r="M5" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N5" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O5" t="str">
+        <v>Estados Unidos</v>
+      </c>
+      <c r="P5" t="str">
+        <v>Paraguay</v>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -820,6 +801,18 @@
       <c r="M6" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N6" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O6" t="str">
+        <v>Haití</v>
+      </c>
+      <c r="P6" t="str">
+        <v>Escocia</v>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -861,6 +854,18 @@
       <c r="M7" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N7" t="str">
+        <v>America/Vancouver</v>
+      </c>
+      <c r="O7" t="str">
+        <v>Australia</v>
+      </c>
+      <c r="P7" t="str">
+        <v>Turquía</v>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -902,6 +907,18 @@
       <c r="M8" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N8" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O8" t="str">
+        <v>Brasil</v>
+      </c>
+      <c r="P8" t="str">
+        <v>Marruecos</v>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -943,6 +960,18 @@
       <c r="M9" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N9" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O9" t="str">
+        <v>Catar</v>
+      </c>
+      <c r="P9" t="str">
+        <v>Suiza</v>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -984,6 +1013,18 @@
       <c r="M10" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N10" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O10" t="str">
+        <v>Costa de Marfil</v>
+      </c>
+      <c r="P10" t="str">
+        <v>Ecuador</v>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -1025,6 +1066,18 @@
       <c r="M11" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N11" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O11" t="str">
+        <v>Alemania</v>
+      </c>
+      <c r="P11" t="str">
+        <v>Curazao</v>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -1066,6 +1119,18 @@
       <c r="M12" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N12" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O12" t="str">
+        <v>Países Bajos</v>
+      </c>
+      <c r="P12" t="str">
+        <v>Japón</v>
+      </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -1107,6 +1172,18 @@
       <c r="M13" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N13" t="str">
+        <v>America/Monterrey</v>
+      </c>
+      <c r="O13" t="str">
+        <v>Suecia</v>
+      </c>
+      <c r="P13" t="str">
+        <v>Túnez</v>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -1148,6 +1225,18 @@
       <c r="M14" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N14" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O14" t="str">
+        <v>Arabia Saudita</v>
+      </c>
+      <c r="P14" t="str">
+        <v>Uruguay</v>
+      </c>
+      <c r="Q14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -1189,6 +1278,18 @@
       <c r="M15" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N15" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O15" t="str">
+        <v>España</v>
+      </c>
+      <c r="P15" t="str">
+        <v>Cabo Verde</v>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -1230,6 +1331,18 @@
       <c r="M16" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N16" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O16" t="str">
+        <v>Irán</v>
+      </c>
+      <c r="P16" t="str">
+        <v>Nueva Zelanda</v>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -1271,6 +1384,18 @@
       <c r="M17" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N17" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O17" t="str">
+        <v>Bélgica</v>
+      </c>
+      <c r="P17" t="str">
+        <v>Egipto</v>
+      </c>
+      <c r="Q17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -1312,6 +1437,18 @@
       <c r="M18" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N18" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O18" t="str">
+        <v>Francia</v>
+      </c>
+      <c r="P18" t="str">
+        <v>Senegal</v>
+      </c>
+      <c r="Q18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -1353,6 +1490,18 @@
       <c r="M19" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N19" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O19" t="str">
+        <v>Irak</v>
+      </c>
+      <c r="P19" t="str">
+        <v>Noruega</v>
+      </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -1394,6 +1543,18 @@
       <c r="M20" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N20" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O20" t="str">
+        <v>Argentina</v>
+      </c>
+      <c r="P20" t="str">
+        <v>Argelia</v>
+      </c>
+      <c r="Q20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -1435,6 +1596,18 @@
       <c r="M21" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N21" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O21" t="str">
+        <v>Austria</v>
+      </c>
+      <c r="P21" t="str">
+        <v>Jordania</v>
+      </c>
+      <c r="Q21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -1476,6 +1649,18 @@
       <c r="M22" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N22" t="str">
+        <v>America/Toronto</v>
+      </c>
+      <c r="O22" t="str">
+        <v>Ghana</v>
+      </c>
+      <c r="P22" t="str">
+        <v>Panamá</v>
+      </c>
+      <c r="Q22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -1517,6 +1702,18 @@
       <c r="M23" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N23" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O23" t="str">
+        <v>Inglaterra</v>
+      </c>
+      <c r="P23" t="str">
+        <v>Croacia</v>
+      </c>
+      <c r="Q23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -1558,6 +1755,18 @@
       <c r="M24" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N24" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O24" t="str">
+        <v>Portugal</v>
+      </c>
+      <c r="P24" t="str">
+        <v>República Democrática del Congo</v>
+      </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -1599,6 +1808,18 @@
       <c r="M25" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N25" t="str">
+        <v>America/Mexico_City</v>
+      </c>
+      <c r="O25" t="str">
+        <v>Uzbekistán</v>
+      </c>
+      <c r="P25" t="str">
+        <v>Colombia</v>
+      </c>
+      <c r="Q25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -1640,6 +1861,18 @@
       <c r="M26" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N26" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O26" t="str">
+        <v>Chequia</v>
+      </c>
+      <c r="P26" t="str">
+        <v>Sudáfrica</v>
+      </c>
+      <c r="Q26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -1681,6 +1914,18 @@
       <c r="M27" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N27" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O27" t="str">
+        <v>Suiza</v>
+      </c>
+      <c r="P27" t="str">
+        <v>Bosnia y Herzegovina</v>
+      </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -1722,6 +1967,18 @@
       <c r="M28" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N28" t="str">
+        <v>America/Vancouver</v>
+      </c>
+      <c r="O28" t="str">
+        <v>Canadá</v>
+      </c>
+      <c r="P28" t="str">
+        <v>Catar</v>
+      </c>
+      <c r="Q28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -1763,6 +2020,18 @@
       <c r="M29" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N29" t="str">
+        <v>America/Mexico_City</v>
+      </c>
+      <c r="O29" t="str">
+        <v>México</v>
+      </c>
+      <c r="P29" t="str">
+        <v>Corea del Sur</v>
+      </c>
+      <c r="Q29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30">
@@ -1804,6 +2073,18 @@
       <c r="M30" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N30" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O30" t="str">
+        <v>Brasil</v>
+      </c>
+      <c r="P30" t="str">
+        <v>Haití</v>
+      </c>
+      <c r="Q30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -1845,6 +2126,18 @@
       <c r="M31" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N31" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O31" t="str">
+        <v>Escocia</v>
+      </c>
+      <c r="P31" t="str">
+        <v>Marruecos</v>
+      </c>
+      <c r="Q31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -1886,6 +2179,18 @@
       <c r="M32" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N32" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O32" t="str">
+        <v>Turquía</v>
+      </c>
+      <c r="P32" t="str">
+        <v>Paraguay</v>
+      </c>
+      <c r="Q32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33">
@@ -1927,6 +2232,18 @@
       <c r="M33" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N33" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O33" t="str">
+        <v>Estados Unidos</v>
+      </c>
+      <c r="P33" t="str">
+        <v>Australia</v>
+      </c>
+      <c r="Q33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -1968,6 +2285,18 @@
       <c r="M34" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N34" t="str">
+        <v>America/Toronto</v>
+      </c>
+      <c r="O34" t="str">
+        <v>Alemania</v>
+      </c>
+      <c r="P34" t="str">
+        <v>Costa de Marfil</v>
+      </c>
+      <c r="Q34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35">
@@ -2009,6 +2338,18 @@
       <c r="M35" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N35" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O35" t="str">
+        <v>Ecuador</v>
+      </c>
+      <c r="P35" t="str">
+        <v>Curazao</v>
+      </c>
+      <c r="Q35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36">
@@ -2050,6 +2391,18 @@
       <c r="M36" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N36" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O36" t="str">
+        <v>Países Bajos</v>
+      </c>
+      <c r="P36" t="str">
+        <v>Suecia</v>
+      </c>
+      <c r="Q36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37">
@@ -2091,6 +2444,18 @@
       <c r="M37" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N37" t="str">
+        <v>America/Monterrey</v>
+      </c>
+      <c r="O37" t="str">
+        <v>Túnez</v>
+      </c>
+      <c r="P37" t="str">
+        <v>Japón</v>
+      </c>
+      <c r="Q37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38">
@@ -2132,6 +2497,18 @@
       <c r="M38" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N38" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O38" t="str">
+        <v>Uruguay</v>
+      </c>
+      <c r="P38" t="str">
+        <v>Cabo Verde</v>
+      </c>
+      <c r="Q38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39">
@@ -2173,6 +2550,18 @@
       <c r="M39" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N39" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O39" t="str">
+        <v>España</v>
+      </c>
+      <c r="P39" t="str">
+        <v>Arabia Saudita</v>
+      </c>
+      <c r="Q39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40">
@@ -2214,6 +2603,18 @@
       <c r="M40" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N40" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O40" t="str">
+        <v>Bélgica</v>
+      </c>
+      <c r="P40" t="str">
+        <v>Irán</v>
+      </c>
+      <c r="Q40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41">
@@ -2255,6 +2656,18 @@
       <c r="M41" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N41" t="str">
+        <v>America/Vancouver</v>
+      </c>
+      <c r="O41" t="str">
+        <v>Nueva Zelanda</v>
+      </c>
+      <c r="P41" t="str">
+        <v>Egipto</v>
+      </c>
+      <c r="Q41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42">
@@ -2296,6 +2709,18 @@
       <c r="M42" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N42" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O42" t="str">
+        <v>Noruega</v>
+      </c>
+      <c r="P42" t="str">
+        <v>Senegal</v>
+      </c>
+      <c r="Q42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43">
@@ -2337,6 +2762,18 @@
       <c r="M43" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N43" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O43" t="str">
+        <v>Francia</v>
+      </c>
+      <c r="P43" t="str">
+        <v>Irak</v>
+      </c>
+      <c r="Q43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44">
@@ -2378,6 +2815,18 @@
       <c r="M44" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N44" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O44" t="str">
+        <v>Argentina</v>
+      </c>
+      <c r="P44" t="str">
+        <v>Austria</v>
+      </c>
+      <c r="Q44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45">
@@ -2419,6 +2868,18 @@
       <c r="M45" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N45" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O45" t="str">
+        <v>Jordania</v>
+      </c>
+      <c r="P45" t="str">
+        <v>Argelia</v>
+      </c>
+      <c r="Q45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46">
@@ -2460,6 +2921,18 @@
       <c r="M46" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N46" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O46" t="str">
+        <v>Inglaterra</v>
+      </c>
+      <c r="P46" t="str">
+        <v>Ghana</v>
+      </c>
+      <c r="Q46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47">
@@ -2501,6 +2974,18 @@
       <c r="M47" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N47" t="str">
+        <v>America/Toronto</v>
+      </c>
+      <c r="O47" t="str">
+        <v>Panamá</v>
+      </c>
+      <c r="P47" t="str">
+        <v>Croacia</v>
+      </c>
+      <c r="Q47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48">
@@ -2542,6 +3027,18 @@
       <c r="M48" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N48" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O48" t="str">
+        <v>Portugal</v>
+      </c>
+      <c r="P48" t="str">
+        <v>Uzbekistán</v>
+      </c>
+      <c r="Q48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49">
@@ -2583,6 +3080,18 @@
       <c r="M49" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N49" t="str">
+        <v>America/Mexico_City</v>
+      </c>
+      <c r="O49" t="str">
+        <v>Colombia</v>
+      </c>
+      <c r="P49" t="str">
+        <v>República Democrática del Congo</v>
+      </c>
+      <c r="Q49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50">
@@ -2624,6 +3133,18 @@
       <c r="M50" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N50" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O50" t="str">
+        <v>Escocia</v>
+      </c>
+      <c r="P50" t="str">
+        <v>Brasil</v>
+      </c>
+      <c r="Q50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51">
@@ -2665,6 +3186,18 @@
       <c r="M51" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N51" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O51" t="str">
+        <v>Marruecos</v>
+      </c>
+      <c r="P51" t="str">
+        <v>Haití</v>
+      </c>
+      <c r="Q51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52">
@@ -2706,6 +3239,18 @@
       <c r="M52" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N52" t="str">
+        <v>America/Vancouver</v>
+      </c>
+      <c r="O52" t="str">
+        <v>Suiza</v>
+      </c>
+      <c r="P52" t="str">
+        <v>Canadá</v>
+      </c>
+      <c r="Q52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53">
@@ -2747,6 +3292,18 @@
       <c r="M53" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N53" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O53" t="str">
+        <v>Bosnia y Herzegovina</v>
+      </c>
+      <c r="P53" t="str">
+        <v>Catar</v>
+      </c>
+      <c r="Q53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54">
@@ -2788,6 +3345,18 @@
       <c r="M54" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N54" t="str">
+        <v>America/Mexico_City</v>
+      </c>
+      <c r="O54" t="str">
+        <v>Chequia</v>
+      </c>
+      <c r="P54" t="str">
+        <v>México</v>
+      </c>
+      <c r="Q54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55">
@@ -2829,6 +3398,18 @@
       <c r="M55" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N55" t="str">
+        <v>America/Monterrey</v>
+      </c>
+      <c r="O55" t="str">
+        <v>Sudáfrica</v>
+      </c>
+      <c r="P55" t="str">
+        <v>Corea del Sur</v>
+      </c>
+      <c r="Q55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56">
@@ -2870,6 +3451,18 @@
       <c r="M56" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N56" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O56" t="str">
+        <v>Curazao</v>
+      </c>
+      <c r="P56" t="str">
+        <v>Costa de Marfil</v>
+      </c>
+      <c r="Q56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57">
@@ -2911,6 +3504,18 @@
       <c r="M57" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N57" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O57" t="str">
+        <v>Ecuador</v>
+      </c>
+      <c r="P57" t="str">
+        <v>Alemania</v>
+      </c>
+      <c r="Q57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58">
@@ -2952,6 +3557,18 @@
       <c r="M58" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N58" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O58" t="str">
+        <v>Japón</v>
+      </c>
+      <c r="P58" t="str">
+        <v>Suecia</v>
+      </c>
+      <c r="Q58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59">
@@ -2993,6 +3610,18 @@
       <c r="M59" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N59" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O59" t="str">
+        <v>Túnez</v>
+      </c>
+      <c r="P59" t="str">
+        <v>Países Bajos</v>
+      </c>
+      <c r="Q59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60">
@@ -3034,6 +3663,18 @@
       <c r="M60" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N60" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O60" t="str">
+        <v>Turquía</v>
+      </c>
+      <c r="P60" t="str">
+        <v>Estados Unidos</v>
+      </c>
+      <c r="Q60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61">
@@ -3075,6 +3716,18 @@
       <c r="M61" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N61" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O61" t="str">
+        <v>Paraguay</v>
+      </c>
+      <c r="P61" t="str">
+        <v>Australia</v>
+      </c>
+      <c r="Q61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62">
@@ -3116,6 +3769,18 @@
       <c r="M62" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N62" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O62" t="str">
+        <v>Noruega</v>
+      </c>
+      <c r="P62" t="str">
+        <v>Francia</v>
+      </c>
+      <c r="Q62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63">
@@ -3157,6 +3822,18 @@
       <c r="M63" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N63" t="str">
+        <v>America/Toronto</v>
+      </c>
+      <c r="O63" t="str">
+        <v>Senegal</v>
+      </c>
+      <c r="P63" t="str">
+        <v>Irak</v>
+      </c>
+      <c r="Q63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64">
@@ -3198,6 +3875,18 @@
       <c r="M64" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N64" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O64" t="str">
+        <v>Egipto</v>
+      </c>
+      <c r="P64" t="str">
+        <v>Irán</v>
+      </c>
+      <c r="Q64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65">
@@ -3239,6 +3928,18 @@
       <c r="M65" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N65" t="str">
+        <v>America/Vancouver</v>
+      </c>
+      <c r="O65" t="str">
+        <v>Nueva Zelanda</v>
+      </c>
+      <c r="P65" t="str">
+        <v>Bélgica</v>
+      </c>
+      <c r="Q65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66">
@@ -3280,6 +3981,18 @@
       <c r="M66" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N66" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O66" t="str">
+        <v>Cabo Verde</v>
+      </c>
+      <c r="P66" t="str">
+        <v>Arabia Saudita</v>
+      </c>
+      <c r="Q66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67">
@@ -3321,6 +4034,18 @@
       <c r="M67" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N67" t="str">
+        <v>America/Mexico_City</v>
+      </c>
+      <c r="O67" t="str">
+        <v>Uruguay</v>
+      </c>
+      <c r="P67" t="str">
+        <v>España</v>
+      </c>
+      <c r="Q67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68">
@@ -3362,6 +4087,18 @@
       <c r="M68" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N68" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O68" t="str">
+        <v>Panamá</v>
+      </c>
+      <c r="P68" t="str">
+        <v>Inglaterra</v>
+      </c>
+      <c r="Q68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69">
@@ -3403,6 +4140,18 @@
       <c r="M69" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N69" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O69" t="str">
+        <v>Croacia</v>
+      </c>
+      <c r="P69" t="str">
+        <v>Ghana</v>
+      </c>
+      <c r="Q69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70">
@@ -3444,6 +4193,18 @@
       <c r="M70" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N70" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O70" t="str">
+        <v>Argelia</v>
+      </c>
+      <c r="P70" t="str">
+        <v>Austria</v>
+      </c>
+      <c r="Q70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71">
@@ -3485,6 +4246,18 @@
       <c r="M71" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N71" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O71" t="str">
+        <v>Jordania</v>
+      </c>
+      <c r="P71" t="str">
+        <v>Argentina</v>
+      </c>
+      <c r="Q71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72">
@@ -3526,6 +4299,18 @@
       <c r="M72" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N72" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O72" t="str">
+        <v>Colombia</v>
+      </c>
+      <c r="P72" t="str">
+        <v>Portugal</v>
+      </c>
+      <c r="Q72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73">
@@ -3567,6 +4352,18 @@
       <c r="M73" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
       </c>
+      <c r="N73" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O73" t="str">
+        <v>República Democrática del Congo</v>
+      </c>
+      <c r="P73" t="str">
+        <v>Uzbekistán</v>
+      </c>
+      <c r="Q73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74">
@@ -3575,9 +4372,6 @@
       <c r="B74" t="str">
         <v>Ronda de 32</v>
       </c>
-      <c r="C74" t="str">
-        <v/>
-      </c>
       <c r="D74" s="1">
         <v>46201</v>
       </c>
@@ -3607,6 +4401,18 @@
       </c>
       <c r="M74" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N74" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O74" t="str">
+        <v>Segundo del Grupo A</v>
+      </c>
+      <c r="P74" t="str">
+        <v>Segundo del Grupo B</v>
+      </c>
+      <c r="Q74" t="str">
+        <v/>
       </c>
     </row>
     <row r="75">
@@ -3616,9 +4422,6 @@
       <c r="B75" t="str">
         <v>Ronda de 32</v>
       </c>
-      <c r="C75" t="str">
-        <v/>
-      </c>
       <c r="D75" s="1">
         <v>46202</v>
       </c>
@@ -3648,6 +4451,18 @@
       </c>
       <c r="M75" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N75" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O75" t="str">
+        <v>Ganador del Grupo E</v>
+      </c>
+      <c r="P75" t="str">
+        <v>Mejor tercero A/B/C/D/F</v>
+      </c>
+      <c r="Q75" t="str">
+        <v/>
       </c>
     </row>
     <row r="76">
@@ -3657,9 +4472,6 @@
       <c r="B76" t="str">
         <v>Ronda de 32</v>
       </c>
-      <c r="C76" t="str">
-        <v/>
-      </c>
       <c r="D76" s="1">
         <v>46202</v>
       </c>
@@ -3689,6 +4501,18 @@
       </c>
       <c r="M76" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N76" t="str">
+        <v>America/Monterrey</v>
+      </c>
+      <c r="O76" t="str">
+        <v>Ganador del Grupo F</v>
+      </c>
+      <c r="P76" t="str">
+        <v>Segundo del Grupo C</v>
+      </c>
+      <c r="Q76" t="str">
+        <v/>
       </c>
     </row>
     <row r="77">
@@ -3698,9 +4522,6 @@
       <c r="B77" t="str">
         <v>Ronda de 32</v>
       </c>
-      <c r="C77" t="str">
-        <v/>
-      </c>
       <c r="D77" s="1">
         <v>46202</v>
       </c>
@@ -3730,6 +4551,18 @@
       </c>
       <c r="M77" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N77" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O77" t="str">
+        <v>Ganador del Grupo C</v>
+      </c>
+      <c r="P77" t="str">
+        <v>Segundo del Grupo F</v>
+      </c>
+      <c r="Q77" t="str">
+        <v/>
       </c>
     </row>
     <row r="78">
@@ -3739,9 +4572,6 @@
       <c r="B78" t="str">
         <v>Ronda de 32</v>
       </c>
-      <c r="C78" t="str">
-        <v/>
-      </c>
       <c r="D78" s="1">
         <v>46203</v>
       </c>
@@ -3771,6 +4601,18 @@
       </c>
       <c r="M78" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N78" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O78" t="str">
+        <v>Ganador del Grupo I</v>
+      </c>
+      <c r="P78" t="str">
+        <v>Mejor tercero C/D/F/G/H</v>
+      </c>
+      <c r="Q78" t="str">
+        <v/>
       </c>
     </row>
     <row r="79">
@@ -3780,9 +4622,6 @@
       <c r="B79" t="str">
         <v>Ronda de 32</v>
       </c>
-      <c r="C79" t="str">
-        <v/>
-      </c>
       <c r="D79" s="1">
         <v>46203</v>
       </c>
@@ -3812,6 +4651,18 @@
       </c>
       <c r="M79" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N79" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O79" t="str">
+        <v>Segundo del Grupo E</v>
+      </c>
+      <c r="P79" t="str">
+        <v>Segundo del Grupo I</v>
+      </c>
+      <c r="Q79" t="str">
+        <v/>
       </c>
     </row>
     <row r="80">
@@ -3821,9 +4672,6 @@
       <c r="B80" t="str">
         <v>Ronda de 32</v>
       </c>
-      <c r="C80" t="str">
-        <v/>
-      </c>
       <c r="D80" s="1">
         <v>46203</v>
       </c>
@@ -3853,6 +4701,18 @@
       </c>
       <c r="M80" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N80" t="str">
+        <v>America/Mexico_City</v>
+      </c>
+      <c r="O80" t="str">
+        <v>Ganador del Grupo A</v>
+      </c>
+      <c r="P80" t="str">
+        <v>Mejor tercero C/E/F/H/I</v>
+      </c>
+      <c r="Q80" t="str">
+        <v/>
       </c>
     </row>
     <row r="81">
@@ -3862,9 +4722,6 @@
       <c r="B81" t="str">
         <v>Ronda de 32</v>
       </c>
-      <c r="C81" t="str">
-        <v/>
-      </c>
       <c r="D81" s="1">
         <v>46204</v>
       </c>
@@ -3894,6 +4751,18 @@
       </c>
       <c r="M81" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N81" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O81" t="str">
+        <v>Ganador del Grupo L</v>
+      </c>
+      <c r="P81" t="str">
+        <v>Mejor tercero E/H/I/J/K</v>
+      </c>
+      <c r="Q81" t="str">
+        <v/>
       </c>
     </row>
     <row r="82">
@@ -3903,9 +4772,6 @@
       <c r="B82" t="str">
         <v>Ronda de 32</v>
       </c>
-      <c r="C82" t="str">
-        <v/>
-      </c>
       <c r="D82" s="1">
         <v>46204</v>
       </c>
@@ -3935,6 +4801,18 @@
       </c>
       <c r="M82" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N82" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O82" t="str">
+        <v>Ganador del Grupo D</v>
+      </c>
+      <c r="P82" t="str">
+        <v>Mejor tercero B/E/F/I/J</v>
+      </c>
+      <c r="Q82" t="str">
+        <v/>
       </c>
     </row>
     <row r="83">
@@ -3944,9 +4822,6 @@
       <c r="B83" t="str">
         <v>Ronda de 32</v>
       </c>
-      <c r="C83" t="str">
-        <v/>
-      </c>
       <c r="D83" s="1">
         <v>46204</v>
       </c>
@@ -3976,6 +4851,18 @@
       </c>
       <c r="M83" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N83" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O83" t="str">
+        <v>Ganador del Grupo G</v>
+      </c>
+      <c r="P83" t="str">
+        <v>Mejor tercero A/E/H/I/J</v>
+      </c>
+      <c r="Q83" t="str">
+        <v/>
       </c>
     </row>
     <row r="84">
@@ -3985,9 +4872,6 @@
       <c r="B84" t="str">
         <v>Ronda de 32</v>
       </c>
-      <c r="C84" t="str">
-        <v/>
-      </c>
       <c r="D84" s="1">
         <v>46205</v>
       </c>
@@ -4017,6 +4901,18 @@
       </c>
       <c r="M84" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N84" t="str">
+        <v>America/Toronto</v>
+      </c>
+      <c r="O84" t="str">
+        <v>Segundo del Grupo K</v>
+      </c>
+      <c r="P84" t="str">
+        <v>Segundo del Grupo L</v>
+      </c>
+      <c r="Q84" t="str">
+        <v/>
       </c>
     </row>
     <row r="85">
@@ -4026,9 +4922,6 @@
       <c r="B85" t="str">
         <v>Ronda de 32</v>
       </c>
-      <c r="C85" t="str">
-        <v/>
-      </c>
       <c r="D85" s="1">
         <v>46205</v>
       </c>
@@ -4058,6 +4951,18 @@
       </c>
       <c r="M85" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N85" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O85" t="str">
+        <v>Ganador del Grupo H</v>
+      </c>
+      <c r="P85" t="str">
+        <v>Segundo del Grupo J</v>
+      </c>
+      <c r="Q85" t="str">
+        <v/>
       </c>
     </row>
     <row r="86">
@@ -4067,9 +4972,6 @@
       <c r="B86" t="str">
         <v>Ronda de 32</v>
       </c>
-      <c r="C86" t="str">
-        <v/>
-      </c>
       <c r="D86" s="1">
         <v>46205</v>
       </c>
@@ -4099,6 +5001,18 @@
       </c>
       <c r="M86" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N86" t="str">
+        <v>America/Vancouver</v>
+      </c>
+      <c r="O86" t="str">
+        <v>Ganador del Grupo B</v>
+      </c>
+      <c r="P86" t="str">
+        <v>Mejor tercero E/F/G/I/J</v>
+      </c>
+      <c r="Q86" t="str">
+        <v/>
       </c>
     </row>
     <row r="87">
@@ -4108,9 +5022,6 @@
       <c r="B87" t="str">
         <v>Ronda de 32</v>
       </c>
-      <c r="C87" t="str">
-        <v/>
-      </c>
       <c r="D87" s="1">
         <v>46206</v>
       </c>
@@ -4140,6 +5051,18 @@
       </c>
       <c r="M87" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N87" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O87" t="str">
+        <v>Ganador del Grupo J</v>
+      </c>
+      <c r="P87" t="str">
+        <v>Segundo del Grupo H</v>
+      </c>
+      <c r="Q87" t="str">
+        <v/>
       </c>
     </row>
     <row r="88">
@@ -4149,9 +5072,6 @@
       <c r="B88" t="str">
         <v>Ronda de 32</v>
       </c>
-      <c r="C88" t="str">
-        <v/>
-      </c>
       <c r="D88" s="1">
         <v>46206</v>
       </c>
@@ -4181,6 +5101,18 @@
       </c>
       <c r="M88" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N88" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O88" t="str">
+        <v>Ganador del Grupo K</v>
+      </c>
+      <c r="P88" t="str">
+        <v>Mejor tercero D/E/I/J/L</v>
+      </c>
+      <c r="Q88" t="str">
+        <v/>
       </c>
     </row>
     <row r="89">
@@ -4190,9 +5122,6 @@
       <c r="B89" t="str">
         <v>Ronda de 32</v>
       </c>
-      <c r="C89" t="str">
-        <v/>
-      </c>
       <c r="D89" s="1">
         <v>46206</v>
       </c>
@@ -4222,6 +5151,18 @@
       </c>
       <c r="M89" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N89" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O89" t="str">
+        <v>Segundo del Grupo D</v>
+      </c>
+      <c r="P89" t="str">
+        <v>Segundo del Grupo G</v>
+      </c>
+      <c r="Q89" t="str">
+        <v/>
       </c>
     </row>
     <row r="90">
@@ -4231,9 +5172,6 @@
       <c r="B90" t="str">
         <v>Octavos de final</v>
       </c>
-      <c r="C90" t="str">
-        <v/>
-      </c>
       <c r="D90" s="1">
         <v>46207</v>
       </c>
@@ -4263,6 +5201,18 @@
       </c>
       <c r="M90" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N90" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O90" t="str">
+        <v>Ganador del Partido 74</v>
+      </c>
+      <c r="P90" t="str">
+        <v>Ganador del Partido 77</v>
+      </c>
+      <c r="Q90" t="str">
+        <v/>
       </c>
     </row>
     <row r="91">
@@ -4272,9 +5222,6 @@
       <c r="B91" t="str">
         <v>Octavos de final</v>
       </c>
-      <c r="C91" t="str">
-        <v/>
-      </c>
       <c r="D91" s="1">
         <v>46207</v>
       </c>
@@ -4304,6 +5251,18 @@
       </c>
       <c r="M91" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N91" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O91" t="str">
+        <v>Ganador del Partido 73</v>
+      </c>
+      <c r="P91" t="str">
+        <v>Ganador del Partido 75</v>
+      </c>
+      <c r="Q91" t="str">
+        <v/>
       </c>
     </row>
     <row r="92">
@@ -4313,9 +5272,6 @@
       <c r="B92" t="str">
         <v>Octavos de final</v>
       </c>
-      <c r="C92" t="str">
-        <v/>
-      </c>
       <c r="D92" s="1">
         <v>46208</v>
       </c>
@@ -4345,6 +5301,18 @@
       </c>
       <c r="M92" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N92" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O92" t="str">
+        <v>Ganador del Partido 76</v>
+      </c>
+      <c r="P92" t="str">
+        <v>Ganador del Partido 78</v>
+      </c>
+      <c r="Q92" t="str">
+        <v/>
       </c>
     </row>
     <row r="93">
@@ -4354,9 +5322,6 @@
       <c r="B93" t="str">
         <v>Octavos de final</v>
       </c>
-      <c r="C93" t="str">
-        <v/>
-      </c>
       <c r="D93" s="1">
         <v>46208</v>
       </c>
@@ -4386,6 +5351,18 @@
       </c>
       <c r="M93" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N93" t="str">
+        <v>America/Mexico_City</v>
+      </c>
+      <c r="O93" t="str">
+        <v>Ganador del Partido 79</v>
+      </c>
+      <c r="P93" t="str">
+        <v>Ganador del Partido 80</v>
+      </c>
+      <c r="Q93" t="str">
+        <v/>
       </c>
     </row>
     <row r="94">
@@ -4395,9 +5372,6 @@
       <c r="B94" t="str">
         <v>Octavos de final</v>
       </c>
-      <c r="C94" t="str">
-        <v/>
-      </c>
       <c r="D94" s="1">
         <v>46209</v>
       </c>
@@ -4427,6 +5401,18 @@
       </c>
       <c r="M94" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N94" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O94" t="str">
+        <v>Ganador del Partido 83</v>
+      </c>
+      <c r="P94" t="str">
+        <v>Ganador del Partido 84</v>
+      </c>
+      <c r="Q94" t="str">
+        <v/>
       </c>
     </row>
     <row r="95">
@@ -4436,9 +5422,6 @@
       <c r="B95" t="str">
         <v>Octavos de final</v>
       </c>
-      <c r="C95" t="str">
-        <v/>
-      </c>
       <c r="D95" s="1">
         <v>46209</v>
       </c>
@@ -4468,6 +5451,18 @@
       </c>
       <c r="M95" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N95" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O95" t="str">
+        <v>Ganador del Partido 81</v>
+      </c>
+      <c r="P95" t="str">
+        <v>Ganador del Partido 82</v>
+      </c>
+      <c r="Q95" t="str">
+        <v/>
       </c>
     </row>
     <row r="96">
@@ -4477,9 +5472,6 @@
       <c r="B96" t="str">
         <v>Octavos de final</v>
       </c>
-      <c r="C96" t="str">
-        <v/>
-      </c>
       <c r="D96" s="1">
         <v>46210</v>
       </c>
@@ -4509,6 +5501,18 @@
       </c>
       <c r="M96" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N96" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O96" t="str">
+        <v>Ganador del Partido 86</v>
+      </c>
+      <c r="P96" t="str">
+        <v>Ganador del Partido 88</v>
+      </c>
+      <c r="Q96" t="str">
+        <v/>
       </c>
     </row>
     <row r="97">
@@ -4518,9 +5522,6 @@
       <c r="B97" t="str">
         <v>Octavos de final</v>
       </c>
-      <c r="C97" t="str">
-        <v/>
-      </c>
       <c r="D97" s="1">
         <v>46210</v>
       </c>
@@ -4550,6 +5551,18 @@
       </c>
       <c r="M97" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N97" t="str">
+        <v>America/Vancouver</v>
+      </c>
+      <c r="O97" t="str">
+        <v>Ganador del Partido 85</v>
+      </c>
+      <c r="P97" t="str">
+        <v>Ganador del Partido 87</v>
+      </c>
+      <c r="Q97" t="str">
+        <v/>
       </c>
     </row>
     <row r="98">
@@ -4559,9 +5572,6 @@
       <c r="B98" t="str">
         <v>Cuartos de final</v>
       </c>
-      <c r="C98" t="str">
-        <v/>
-      </c>
       <c r="D98" s="1">
         <v>46212</v>
       </c>
@@ -4591,6 +5601,18 @@
       </c>
       <c r="M98" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N98" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O98" t="str">
+        <v>Ganador del Partido 89</v>
+      </c>
+      <c r="P98" t="str">
+        <v>Ganador del Partido 90</v>
+      </c>
+      <c r="Q98" t="str">
+        <v/>
       </c>
     </row>
     <row r="99">
@@ -4600,9 +5622,6 @@
       <c r="B99" t="str">
         <v>Cuartos de final</v>
       </c>
-      <c r="C99" t="str">
-        <v/>
-      </c>
       <c r="D99" s="1">
         <v>46213</v>
       </c>
@@ -4632,6 +5651,18 @@
       </c>
       <c r="M99" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N99" t="str">
+        <v>America/Los_Angeles</v>
+      </c>
+      <c r="O99" t="str">
+        <v>Ganador del Partido 93</v>
+      </c>
+      <c r="P99" t="str">
+        <v>Ganador del Partido 94</v>
+      </c>
+      <c r="Q99" t="str">
+        <v/>
       </c>
     </row>
     <row r="100">
@@ -4641,9 +5672,6 @@
       <c r="B100" t="str">
         <v>Cuartos de final</v>
       </c>
-      <c r="C100" t="str">
-        <v/>
-      </c>
       <c r="D100" s="1">
         <v>46214</v>
       </c>
@@ -4673,6 +5701,18 @@
       </c>
       <c r="M100" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N100" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O100" t="str">
+        <v>Ganador del Partido 91</v>
+      </c>
+      <c r="P100" t="str">
+        <v>Ganador del Partido 92</v>
+      </c>
+      <c r="Q100" t="str">
+        <v/>
       </c>
     </row>
     <row r="101">
@@ -4682,9 +5722,6 @@
       <c r="B101" t="str">
         <v>Cuartos de final</v>
       </c>
-      <c r="C101" t="str">
-        <v/>
-      </c>
       <c r="D101" s="1">
         <v>46214</v>
       </c>
@@ -4714,6 +5751,18 @@
       </c>
       <c r="M101" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N101" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O101" t="str">
+        <v>Ganador del Partido 95</v>
+      </c>
+      <c r="P101" t="str">
+        <v>Ganador del Partido 96</v>
+      </c>
+      <c r="Q101" t="str">
+        <v/>
       </c>
     </row>
     <row r="102">
@@ -4723,9 +5772,6 @@
       <c r="B102" t="str">
         <v>Semifinal</v>
       </c>
-      <c r="C102" t="str">
-        <v/>
-      </c>
       <c r="D102" s="1">
         <v>46217</v>
       </c>
@@ -4755,6 +5801,18 @@
       </c>
       <c r="M102" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N102" t="str">
+        <v>America/Chicago</v>
+      </c>
+      <c r="O102" t="str">
+        <v>Ganador del Partido 97</v>
+      </c>
+      <c r="P102" t="str">
+        <v>Ganador del Partido 98</v>
+      </c>
+      <c r="Q102" t="str">
+        <v/>
       </c>
     </row>
     <row r="103">
@@ -4764,9 +5822,6 @@
       <c r="B103" t="str">
         <v>Semifinal</v>
       </c>
-      <c r="C103" t="str">
-        <v/>
-      </c>
       <c r="D103" s="1">
         <v>46218</v>
       </c>
@@ -4796,6 +5851,18 @@
       </c>
       <c r="M103" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N103" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O103" t="str">
+        <v>Ganador del Partido 99</v>
+      </c>
+      <c r="P103" t="str">
+        <v>Ganador del Partido 100</v>
+      </c>
+      <c r="Q103" t="str">
+        <v/>
       </c>
     </row>
     <row r="104">
@@ -4805,9 +5872,6 @@
       <c r="B104" t="str">
         <v>Tercer puesto</v>
       </c>
-      <c r="C104" t="str">
-        <v/>
-      </c>
       <c r="D104" s="1">
         <v>46221</v>
       </c>
@@ -4837,6 +5901,18 @@
       </c>
       <c r="M104" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N104" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O104" t="str">
+        <v>Perdedor del Partido 101</v>
+      </c>
+      <c r="P104" t="str">
+        <v>Perdedor del Partido 102</v>
+      </c>
+      <c r="Q104" t="str">
+        <v/>
       </c>
     </row>
     <row r="105">
@@ -4846,9 +5922,6 @@
       <c r="B105" t="str">
         <v>Final</v>
       </c>
-      <c r="C105" t="str">
-        <v/>
-      </c>
       <c r="D105" s="1">
         <v>46222</v>
       </c>
@@ -4878,19 +5951,31 @@
       </c>
       <c r="M105" t="str">
         <v>https://www.fifa.com/en/tournaments/mens/worldcup/canadamexicousa2026/scores-fixtures</v>
+      </c>
+      <c r="N105" t="str">
+        <v>America/New_York</v>
+      </c>
+      <c r="O105" t="str">
+        <v>Ganador del Partido 101</v>
+      </c>
+      <c r="P105" t="str">
+        <v>Ganador del Partido 102</v>
+      </c>
+      <c r="Q105" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M105"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q105"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:F2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4903,50 +5988,38 @@
         <v>partido_id</v>
       </c>
       <c r="D1" t="str">
-        <v>goles_local</v>
+        <v>seleccion</v>
       </c>
       <c r="E1" t="str">
-        <v>goles_visitante</v>
+        <v>creado_en</v>
       </c>
       <c r="F1" t="str">
-        <v>puntos_obtenidos</v>
-      </c>
-      <c r="G1" t="str">
-        <v>creado_en</v>
-      </c>
-      <c r="H1" t="str">
         <v>actualizado_en</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>546805bf-d52c-4ab3-96f1-8186074e4dec</v>
+        <v>f6fe23c1-d4c0-47ec-908f-13805de52867</v>
       </c>
       <c r="B2" t="str">
-        <v>c3e0cf6c-33b8-4e0d-a3f3-5221cb4ebc3e</v>
+        <v>USR-DEMO-001</v>
       </c>
       <c r="C2" t="str">
         <v>5</v>
       </c>
-      <c r="D2">
-        <v>3</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2" t="str">
-        <v>2026-06-13T18:57:15.419Z</v>
-      </c>
-      <c r="H2" t="str">
-        <v>2026-06-13T18:57:15.419Z</v>
+      <c r="D2" t="str">
+        <v>empate</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-06-13T19:46:14.630Z</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2026-06-13T19:46:14.630Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4968,57 +6041,57 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>nombre_aplicacion</v>
+        <v>modo</v>
       </c>
       <c r="B2" t="str">
-        <v>ChikiPronósticos</v>
+        <v>encuesta_familiar</v>
       </c>
       <c r="C2" t="str">
-        <v>Nombre visible de la quiniela familiar</v>
+        <v>Elecciones sociales sin premios, pagos ni puntuación por aciertos.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>puntos_marcador_exacto</v>
-      </c>
-      <c r="B3">
-        <v>3</v>
+        <v>opciones</v>
+      </c>
+      <c r="B3" t="str">
+        <v>local|empate|visitante</v>
       </c>
       <c r="C3" t="str">
-        <v>Puntos por acertar el marcador exacto</v>
+        <v>Opciones disponibles por partido.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>puntos_resultado</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
+        <v>bloqueo</v>
+      </c>
+      <c r="B4" t="str">
+        <v>hora_inicio</v>
       </c>
       <c r="C4" t="str">
-        <v>Puntos por acertar ganador o empate</v>
+        <v>La encuesta se cierra automáticamente al comenzar el partido.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>puntos_error</v>
-      </c>
-      <c r="B5">
-        <v>0</v>
+        <v>zona_visualizacion</v>
+      </c>
+      <c r="B5" t="str">
+        <v>America/Lima</v>
       </c>
       <c r="C5" t="str">
-        <v>Puntos cuando no se acierta</v>
+        <v>Todas las fechas se muestran en hora de Lima, Perú.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>zona_horaria_visual</v>
+        <v>avance_llaves</v>
       </c>
       <c r="B6" t="str">
-        <v>America/Lima</v>
+        <v>automatico</v>
       </c>
       <c r="C6" t="str">
-        <v>Zona horaria sugerida para la interfaz</v>
+        <v>Ganadores y perdedores alimentan las siguientes rondas eliminatorias.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>